<commit_message>
Project Atlas v2.15 controlled real batch send readiness
</commit_message>
<xml_diff>
--- a/demo-files/certificate-data-controlled-batch-v215.xlsx
+++ b/demo-files/certificate-data-controlled-batch-v215.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\codex project\Marketing\Project_Atlas\demo-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A67AA786-5719-4C31-BF5E-A426DEF4664E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62BB40AF-4535-4F26-9312-BAB58E3443AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -73,32 +73,37 @@
     <t>AR-CERT-V215-005</t>
   </si>
   <si>
-    <t>test1@example.com</t>
-  </si>
-  <si>
-    <t>test2@example.com</t>
-  </si>
-  <si>
-    <t>test3@example.com</t>
-  </si>
-  <si>
-    <t>test4@example.com</t>
-  </si>
-  <si>
-    <t>test5@example.com</t>
+    <t>aaryarushi7+test1@gmail.com</t>
+  </si>
+  <si>
+    <t>aaryarushi7+test2@gmail.com</t>
+  </si>
+  <si>
+    <t>aaryarushi7+test3@gmail.com</t>
+  </si>
+  <si>
+    <t>aaryarushi7+test4@gmail.com</t>
+  </si>
+  <si>
+    <t>aaryarushi7+test5@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -121,8 +126,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -462,14 +470,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="4" max="4" width="22.69921875" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15.6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -486,7 +494,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="15.6">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -503,7 +511,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="15.6">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -520,7 +528,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="15.6">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -537,7 +545,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="15.6">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -554,7 +562,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="15.6">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -567,12 +575,14 @@
       <c r="D6" t="s">
         <v>16</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="1" t="s">
         <v>21</v>
       </c>
     </row>
+    <row r="7" spans="1:5" ht="15.6"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
     <ignoredError sqref="A1:E1 A6:D6 A2:D2 A3:D3 A4:D4 A5:D5" numberStoredAsText="1"/>
   </ignoredErrors>

</xml_diff>